<commit_message>
feat: make bulk price periods safe
</commit_message>
<xml_diff>
--- a/v3_backend/static/templates/product_upload_template.xlsx
+++ b/v3_backend/static/templates/product_upload_template.xlsx
@@ -329,20 +329,6 @@
 示例: Washington, USA</t>
       </text>
     </comment>
-    <comment ref="T1" authorId="0" shapeId="0">
-      <text>
-        <t>产品有效开始日期
-字段名: effective_from
-示例: 2026-01-01</t>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0" shapeId="0">
-      <text>
-        <t>产品有效结束日期
-字段名: effective_to
-示例: 2026-12-31</t>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
@@ -636,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U4"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -658,8 +644,6 @@
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
     <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -758,16 +742,6 @@
           <t>country_of_origin</t>
         </is>
       </c>
-      <c r="T1" s="2" t="inlineStr">
-        <is>
-          <t>effective_from</t>
-        </is>
-      </c>
-      <c r="U1" s="2" t="inlineStr">
-        <is>
-          <t>effective_to</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -852,12 +826,6 @@
         <is>
           <t>Washington, USA</t>
         </is>
-      </c>
-      <c r="T2" s="6" t="n">
-        <v>46023</v>
-      </c>
-      <c r="U2" s="6" t="n">
-        <v>46387</v>
       </c>
     </row>
     <row r="3">
@@ -936,8 +904,6 @@
           <t>Japan</t>
         </is>
       </c>
-      <c r="T3" s="6" t="n"/>
-      <c r="U3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -971,8 +937,6 @@
       <c r="Q4" s="3" t="n"/>
       <c r="R4" s="3" t="n"/>
       <c r="S4" s="3" t="n"/>
-      <c r="T4" s="6" t="n"/>
-      <c r="U4" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -986,7 +950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1382,7 +1346,7 @@
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>采购价开始生效的日期。新产品空 = 不限制起始；更新时空 = 保留旧值。</t>
+          <t>采购价开始生效的日期。留空表示本行不新建期间；更新时空 = 保留旧值。</t>
         </is>
       </c>
     </row>
@@ -1409,7 +1373,7 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>采购价有效的最后一天。新产品空 = 不限制结束；更新时空 = 保留旧值。</t>
+          <t>采购价有效的最后一天。一个期间必须同时填写开始和结束日期。</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1427,7 @@
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>卖价开始生效的日期。新产品空 = 不限制起始；更新时空 = 保留旧值。</t>
+          <t>卖价开始生效的日期。留空表示本行不新建期间；更新时空 = 保留旧值。</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1454,7 @@
       </c>
       <c r="E30" s="10" t="inlineStr">
         <is>
-          <t>卖价有效的最后一天。新产品空 = 不限制结束；更新时空 = 保留旧值。</t>
+          <t>卖价有效的最后一天。一个期间必须同时填写开始和结束日期。</t>
         </is>
       </c>
     </row>
@@ -1629,294 +1593,240 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="60" customHeight="1">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>effective_from</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>可选</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>日期 YYYY-MM-DD</t>
-        </is>
-      </c>
-      <c r="E36" s="10" t="inlineStr">
-        <is>
-          <t>控制产品本身是否可用于匹配，不代表采购价或卖价有效期。新产品空 = 不限制起始；更新时空 = 保留旧值。</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="60" customHeight="1">
-      <c r="A37" s="9" t="inlineStr">
-        <is>
-          <t>effective_to</t>
-        </is>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>可选</t>
-        </is>
-      </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="inlineStr">
-        <is>
-          <t>日期 YYYY-MM-DD</t>
-        </is>
-      </c>
-      <c r="E37" s="10" t="inlineStr">
-        <is>
-          <t>控制产品本身是否可用于匹配，不代表采购价或卖价有效期。新产品空 = 不限制结束；更新时空 = 保留旧值。</t>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—— 外键字段填名字（不是 ID）—— </t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>类别 / 供应商 / 国家 / 港口 这 4 个字段，请填**名称**：</t>
         </is>
       </c>
     </row>
     <row r="40" ht="30" customHeight="1">
-      <c r="A40" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">—— 外键字段填名字（不是 ID）—— </t>
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · 类别 → 在「数据管理」→「类别」Tab 看完整列表（例：FRUIT, DAIRY, MEAT）</t>
         </is>
       </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>类别 / 供应商 / 国家 / 港口 这 4 个字段，请填**名称**：</t>
+          <t xml:space="preserve">  · 供应商 → 「供应商」Tab（例：Sunkist Growers Inc.）</t>
         </is>
       </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · 类别 → 在「数据管理」→「类别」Tab 看完整列表（例：FRUIT, DAIRY, MEAT）</t>
+          <t xml:space="preserve">  · 国家 → 「国家」Tab（例：USA, Japan, Australia）</t>
         </is>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · 供应商 → 「供应商」Tab（例：Sunkist Growers Inc.）</t>
+          <t xml:space="preserve">  · 港口 → 「港口」Tab（例：Yokohama, Hong Kong）</t>
         </is>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · 国家 → 「国家」Tab（例：USA, Japan, Australia）</t>
+          <t>系统会按这些表的 `name` 字段精确匹配，不区分大小写，自动忽略首尾空格。</t>
         </is>
       </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · 港口 → 「港口」Tab（例：Yokohama, Hong Kong）</t>
+          <t>找不到名字 → 该行会被标记错误，AI 助手会告诉你哪些名字写错了。</t>
         </is>
       </c>
     </row>
     <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>系统会按这些表的 `name` 字段精确匹配，不区分大小写，自动忽略首尾空格。</t>
-        </is>
-      </c>
+      <c r="A46" s="8" t="inlineStr"/>
     </row>
     <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>找不到名字 → 该行会被标记错误，AI 助手会告诉你哪些名字写错了。</t>
+      <c r="A47" s="11" t="inlineStr">
+        <is>
+          <t>—— 常见错误 ——</t>
         </is>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="8" t="inlineStr"/>
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>1. 把 product_code 改成数字格式 → 00100 变成 100 → 系统找不到已有产品。用文本格式（模板已经设好）。</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="30" customHeight="1">
-      <c r="A49" s="11" t="inlineStr">
-        <is>
-          <t>—— 常见错误 ——</t>
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>2. 采购价 price、卖价 contract_price 填非负数字；超过两位小数按四舍五入处理，0 有效；公式请先粘贴为数值。</t>
         </is>
       </c>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>1. 把 product_code 改成数字格式 → 00100 变成 100 → 系统找不到已有产品。用文本格式（模板已经设好）。</t>
+          <t>3. 国家填 "美国" 但 countries 表里只有 "USA" → 不命中。先去「数据管理」</t>
         </is>
       </c>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>2. 采购价 price、卖价 contract_price 填非负数字；超过两位小数按四舍五入处理，0 有效；公式请先粘贴为数值。</t>
+          <t>查看真实存在的名字。</t>
         </is>
       </c>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>3. 国家填 "美国" 但 countries 表里只有 "USA" → 不命中。先去「数据管理」</t>
+          <t>4. 第 1 行表头改名 / 删列 → 系统识别不到字段。建议保留规范表头；必填列不能删除。</t>
         </is>
       </c>
     </row>
     <row r="53" ht="30" customHeight="1">
-      <c r="A53" s="8" t="inlineStr">
-        <is>
-          <t>查看真实存在的名字。</t>
-        </is>
-      </c>
+      <c r="A53" s="8" t="inlineStr"/>
     </row>
     <row r="54" ht="30" customHeight="1">
-      <c r="A54" s="8" t="inlineStr">
-        <is>
-          <t>4. 第 1 行表头改名 / 删列 → 系统识别不到字段。建议保留规范表头；必填列不能删除。</t>
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>—— 日期格式 ——</t>
         </is>
       </c>
     </row>
     <row r="55" ht="30" customHeight="1">
-      <c r="A55" s="8" t="inlineStr"/>
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>采购价和卖价的有效日期列接受：</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="30" customHeight="1">
-      <c r="A56" s="11" t="inlineStr">
-        <is>
-          <t>—— 日期格式 ——</t>
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · 2026-01-01 （推荐）</t>
         </is>
       </c>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>采购价、卖价和产品本身的所有有效日期列接受：</t>
+          <t xml:space="preserve">  · 2026/01/01</t>
         </is>
       </c>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · 2026-01-01 （推荐）</t>
+          <t xml:space="preserve">  · 2026.01.01</t>
         </is>
       </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · 2026/01/01</t>
+          <t>Excel 把日期单元格存成日期类型也可以，系统会自动转换。</t>
         </is>
       </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · 2026.01.01</t>
+          <t>采购价和卖价各自的开始日期不能晚于各自的结束日期。</t>
         </is>
       </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>Excel 把日期单元格存成日期类型也可以，系统会自动转换。</t>
+          <t>同一商品可以用多行填写多个不重叠的价格期间；相同或重叠区间会在预览阶段报错。</t>
         </is>
       </c>
     </row>
     <row r="62" ht="30" customHeight="1">
-      <c r="A62" s="8" t="inlineStr">
-        <is>
-          <t>采购价和卖价各自的开始日期不能晚于各自的结束日期。</t>
-        </is>
-      </c>
+      <c r="A62" s="8" t="inlineStr"/>
     </row>
     <row r="63" ht="30" customHeight="1">
-      <c r="A63" s="8" t="inlineStr">
-        <is>
-          <t>effective_from / effective_to 是产品整体有效期，不替代两种价格的有效期。</t>
+      <c r="A63" s="11" t="inlineStr">
+        <is>
+          <t>—— 系统不批量管理的字段 ——</t>
         </is>
       </c>
     </row>
     <row r="64" ht="30" customHeight="1">
-      <c r="A64" s="8" t="inlineStr"/>
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>下列字段不会被本模板更新，请通过单条编辑修改：</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="30" customHeight="1">
-      <c r="A65" s="11" t="inlineStr">
-        <is>
-          <t>—— 系统不批量管理的字段 ——</t>
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · status（启用 / 停用）</t>
         </is>
       </c>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>下列字段不会被本模板更新，请通过单条编辑修改：</t>
+          <t xml:space="preserve">  · 历史价格记录（系统会保留 ChangeLog，不在本模板里管）</t>
         </is>
       </c>
     </row>
     <row r="67" ht="30" customHeight="1">
-      <c r="A67" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · status（启用 / 停用）</t>
-        </is>
-      </c>
+      <c r="A67" s="8" t="inlineStr"/>
     </row>
     <row r="68" ht="30" customHeight="1">
-      <c r="A68" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · 历史价格记录（系统会保留 ChangeLog，不在本模板里管）</t>
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>—— 如何修正错误 ——</t>
         </is>
       </c>
     </row>
     <row r="69" ht="30" customHeight="1">
-      <c r="A69" s="8" t="inlineStr"/>
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>AI 助手在 preview 阶段会告诉你每一行的错误。可以：</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="30" customHeight="1">
-      <c r="A70" s="11" t="inlineStr">
-        <is>
-          <t>—— 如何修正错误 ——</t>
+      <c r="A70" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  · 修正 Excel 重新上传</t>
         </is>
       </c>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>AI 助手在 preview 阶段会告诉你每一行的错误。可以：</t>
+          <t xml:space="preserve">  · 或者将可选字段留空后重新上传（必填字段不能留空；空白保留旧值）</t>
         </is>
       </c>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  · 修正 Excel 重新上传</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="30" customHeight="1">
-      <c r="A73" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  · 或者将可选字段留空后重新上传（必填字段不能留空；空白保留旧值）</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="30" customHeight="1">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
           <t xml:space="preserve">  · 或者输入「取消」放弃这个 batch</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="50">
+    <mergeCell ref="A39:E39"/>
     <mergeCell ref="A59:E59"/>
     <mergeCell ref="A48:E48"/>
-    <mergeCell ref="A73:E73"/>
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A64:E64"/>
     <mergeCell ref="A60:E60"/>
@@ -1935,7 +1845,6 @@
     <mergeCell ref="A41:E41"/>
     <mergeCell ref="A46:E46"/>
     <mergeCell ref="A66:E66"/>
-    <mergeCell ref="A74:E74"/>
     <mergeCell ref="A56:E56"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A55:E55"/>
@@ -1953,6 +1862,7 @@
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A62:E62"/>
     <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A38:E38"/>
     <mergeCell ref="A72:E72"/>
     <mergeCell ref="A52:E52"/>
     <mergeCell ref="A10:E10"/>

</xml_diff>